<commit_message>
update (large dump since it's been awhile)
</commit_message>
<xml_diff>
--- a/pseudodata/1000.xlsx
+++ b/pseudodata/1000.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P22"/>
+  <dimension ref="A1:P18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -536,24 +536,24 @@
         <v>0.1</v>
       </c>
       <c r="I2" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>cos(phi_Dp)</t>
+          <t>ALL</t>
         </is>
       </c>
       <c r="K2" t="n">
         <v>100</v>
       </c>
       <c r="L2" t="n">
-        <v>-0.003175054521221397</v>
+        <v>-0.0006411002443443207</v>
       </c>
       <c r="M2" t="n">
-        <v>0.0002652603912890343</v>
+        <v>0.0003614296390853656</v>
       </c>
       <c r="N2" t="n">
-        <v>-0.0001587527260610698</v>
+        <v>-3.205501221721604e-05</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -590,24 +590,24 @@
         <v>0.1</v>
       </c>
       <c r="I3" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>cos(phi_Dp)</t>
+          <t>ALL</t>
         </is>
       </c>
       <c r="K3" t="n">
         <v>100</v>
       </c>
       <c r="L3" t="n">
-        <v>-0.003013416581336232</v>
+        <v>-0.0008634859872505839</v>
       </c>
       <c r="M3" t="n">
-        <v>0.0003575664290226753</v>
+        <v>0.0003680896850621407</v>
       </c>
       <c r="N3" t="n">
-        <v>-0.0001506708290668116</v>
+        <v>-4.317429936252919e-05</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -644,24 +644,24 @@
         <v>0.1</v>
       </c>
       <c r="I4" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>cos(phi_Dp)</t>
+          <t>ALL</t>
         </is>
       </c>
       <c r="K4" t="n">
         <v>100</v>
       </c>
       <c r="L4" t="n">
-        <v>-0.001904625202283462</v>
+        <v>-0.001123042542067654</v>
       </c>
       <c r="M4" t="n">
-        <v>0.0005040356188673103</v>
+        <v>0.0004026693004854471</v>
       </c>
       <c r="N4" t="n">
-        <v>-9.523126011417312e-05</v>
+        <v>-5.615212710338271e-05</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -698,24 +698,24 @@
         <v>0.1</v>
       </c>
       <c r="I5" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>cos(phi_Dp)</t>
+          <t>ALL</t>
         </is>
       </c>
       <c r="K5" t="n">
         <v>100</v>
       </c>
       <c r="L5" t="n">
-        <v>-0.000139728564480392</v>
+        <v>-0.001461251073788138</v>
       </c>
       <c r="M5" t="n">
-        <v>0.0007184779930692618</v>
+        <v>0.0004685761247997976</v>
       </c>
       <c r="N5" t="n">
-        <v>-6.986428224019599e-06</v>
+        <v>-7.306255368940689e-05</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -752,24 +752,24 @@
         <v>0.1</v>
       </c>
       <c r="I6" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>cos(phi_Dp)</t>
+          <t>ALL</t>
         </is>
       </c>
       <c r="K6" t="n">
         <v>100</v>
       </c>
       <c r="L6" t="n">
-        <v>0.002063196833468931</v>
+        <v>-0.001930657635087965</v>
       </c>
       <c r="M6" t="n">
-        <v>0.001023477386483585</v>
+        <v>0.0005736112390174919</v>
       </c>
       <c r="N6" t="n">
-        <v>0.0001031598416734466</v>
+        <v>-9.653288175439826e-05</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -806,24 +806,24 @@
         <v>0.1</v>
       </c>
       <c r="I7" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>cos(phi_Dp)</t>
+          <t>ALL</t>
         </is>
       </c>
       <c r="K7" t="n">
         <v>100</v>
       </c>
       <c r="L7" t="n">
-        <v>0.004523445992083649</v>
+        <v>-0.002591332123535291</v>
       </c>
       <c r="M7" t="n">
-        <v>0.001419320114396683</v>
+        <v>0.0007294971280996292</v>
       </c>
       <c r="N7" t="n">
-        <v>0.0002261722996041825</v>
+        <v>-0.0001295666061767646</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -860,24 +860,24 @@
         <v>0.1</v>
       </c>
       <c r="I8" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>cos(phi_Dp)</t>
+          <t>ALL</t>
         </is>
       </c>
       <c r="K8" t="n">
         <v>100</v>
       </c>
       <c r="L8" t="n">
-        <v>0.006880287888113445</v>
+        <v>-0.00350612702292311</v>
       </c>
       <c r="M8" t="n">
-        <v>0.0018714884429574</v>
+        <v>0.000951605582013245</v>
       </c>
       <c r="N8" t="n">
-        <v>0.0003440143944056723</v>
+        <v>-0.0001753063511461555</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -908,30 +908,30 @@
         <v>0.5</v>
       </c>
       <c r="G9" t="n">
-        <v>2</v>
+        <v>5.5</v>
       </c>
       <c r="H9" t="n">
         <v>0.1</v>
       </c>
       <c r="I9" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>cos(phi_Dp)cos(phi_kp)</t>
+          <t>ALL</t>
         </is>
       </c>
       <c r="K9" t="n">
         <v>100</v>
       </c>
       <c r="L9" t="n">
-        <v>-0.001087930007562636</v>
+        <v>-0.004738003889388833</v>
       </c>
       <c r="M9" t="n">
-        <v>0.0002652603912890343</v>
+        <v>0.001259129789717481</v>
       </c>
       <c r="N9" t="n">
-        <v>-5.439650037813182e-05</v>
+        <v>-0.0002369001944694416</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -962,30 +962,30 @@
         <v>0.5</v>
       </c>
       <c r="G10" t="n">
-        <v>2.5</v>
+        <v>6</v>
       </c>
       <c r="H10" t="n">
         <v>0.1</v>
       </c>
       <c r="I10" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>cos(phi_Dp)cos(phi_kp)</t>
+          <t>ALL</t>
         </is>
       </c>
       <c r="K10" t="n">
         <v>100</v>
       </c>
       <c r="L10" t="n">
-        <v>-0.001556887859018811</v>
+        <v>-0.006355961735605872</v>
       </c>
       <c r="M10" t="n">
-        <v>0.0003575664290226753</v>
+        <v>0.001675649786666132</v>
       </c>
       <c r="N10" t="n">
-        <v>-7.784439295094058e-05</v>
+        <v>-0.0003177980867802937</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1016,30 +1016,30 @@
         <v>0.5</v>
       </c>
       <c r="G11" t="n">
-        <v>3</v>
+        <v>6.5</v>
       </c>
       <c r="H11" t="n">
         <v>0.1</v>
       </c>
       <c r="I11" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>cos(phi_Dp)cos(phi_kp)</t>
+          <t>ALL</t>
         </is>
       </c>
       <c r="K11" t="n">
         <v>100</v>
       </c>
       <c r="L11" t="n">
-        <v>-0.001541633237940651</v>
+        <v>-0.008447143432763825</v>
       </c>
       <c r="M11" t="n">
-        <v>0.0005040356188673103</v>
+        <v>0.002227087166477917</v>
       </c>
       <c r="N11" t="n">
-        <v>-7.708166189703256e-05</v>
+        <v>-0.0004223571716381913</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1070,30 +1070,30 @@
         <v>0.5</v>
       </c>
       <c r="G12" t="n">
-        <v>3.5</v>
+        <v>7</v>
       </c>
       <c r="H12" t="n">
         <v>0.1</v>
       </c>
       <c r="I12" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>cos(phi_Dp)cos(phi_kp)</t>
+          <t>ALL</t>
         </is>
       </c>
       <c r="K12" t="n">
         <v>100</v>
       </c>
       <c r="L12" t="n">
-        <v>-0.001069757943046558</v>
+        <v>-0.01110350173622898</v>
       </c>
       <c r="M12" t="n">
-        <v>0.0007184779930692618</v>
+        <v>0.00293069039784746</v>
       </c>
       <c r="N12" t="n">
-        <v>-5.348789715232792e-05</v>
+        <v>-0.0005551750868114489</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1124,30 +1124,30 @@
         <v>0.5</v>
       </c>
       <c r="G13" t="n">
-        <v>4</v>
+        <v>7.5</v>
       </c>
       <c r="H13" t="n">
         <v>0.1</v>
       </c>
       <c r="I13" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>cos(phi_Dp)cos(phi_kp)</t>
+          <t>ALL</t>
         </is>
       </c>
       <c r="K13" t="n">
         <v>100</v>
       </c>
       <c r="L13" t="n">
-        <v>-0.0002841322889191621</v>
+        <v>-0.0143311444809686</v>
       </c>
       <c r="M13" t="n">
-        <v>0.001023477386483585</v>
+        <v>0.003775894295266418</v>
       </c>
       <c r="N13" t="n">
-        <v>-1.420661444595811e-05</v>
+        <v>-0.00071655722404843</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1178,30 +1178,30 @@
         <v>0.5</v>
       </c>
       <c r="G14" t="n">
-        <v>4.5</v>
+        <v>8</v>
       </c>
       <c r="H14" t="n">
         <v>0.1</v>
       </c>
       <c r="I14" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>cos(phi_Dp)cos(phi_kp)</t>
+          <t>ALL</t>
         </is>
       </c>
       <c r="K14" t="n">
         <v>100</v>
       </c>
       <c r="L14" t="n">
-        <v>0.0006551662909760984</v>
+        <v>-0.0179414341322815</v>
       </c>
       <c r="M14" t="n">
-        <v>0.001419320114396683</v>
+        <v>0.004725268689439141</v>
       </c>
       <c r="N14" t="n">
-        <v>3.275831454880492e-05</v>
+        <v>-0.0008970717066140752</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1232,30 +1232,30 @@
         <v>0.5</v>
       </c>
       <c r="G15" t="n">
-        <v>5</v>
+        <v>8.5</v>
       </c>
       <c r="H15" t="n">
         <v>0.1</v>
       </c>
       <c r="I15" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>cos(phi_Dp)cos(phi_kp)</t>
+          <t>ALL</t>
         </is>
       </c>
       <c r="K15" t="n">
         <v>100</v>
       </c>
       <c r="L15" t="n">
-        <v>0.001693601273389158</v>
+        <v>-0.02168739987944248</v>
       </c>
       <c r="M15" t="n">
-        <v>0.0018714884429574</v>
+        <v>0.005766904173553507</v>
       </c>
       <c r="N15" t="n">
-        <v>8.468006366945793e-05</v>
+        <v>-0.001084369993972124</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1286,30 +1286,30 @@
         <v>0.5</v>
       </c>
       <c r="G16" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="H16" t="n">
         <v>0.1</v>
       </c>
       <c r="I16" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>sin(phi_Dp)sin(phi_kp)</t>
+          <t>ALL</t>
         </is>
       </c>
       <c r="K16" t="n">
         <v>100</v>
       </c>
       <c r="L16" t="n">
-        <v>0.0002242848669054327</v>
+        <v>-0.02561778505888466</v>
       </c>
       <c r="M16" t="n">
-        <v>0.0002652603912890343</v>
+        <v>0.006965783251712316</v>
       </c>
       <c r="N16" t="n">
-        <v>1.121424334527164e-05</v>
+        <v>-0.001280889252944233</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -1340,30 +1340,30 @@
         <v>0.5</v>
       </c>
       <c r="G17" t="n">
-        <v>2.5</v>
+        <v>9.5</v>
       </c>
       <c r="H17" t="n">
         <v>0.1</v>
       </c>
       <c r="I17" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>sin(phi_Dp)sin(phi_kp)</t>
+          <t>ALL</t>
         </is>
       </c>
       <c r="K17" t="n">
         <v>100</v>
       </c>
       <c r="L17" t="n">
-        <v>4.711452495812959e-05</v>
+        <v>-0.03014863330692746</v>
       </c>
       <c r="M17" t="n">
-        <v>0.0003575664290226753</v>
+        <v>0.008427225954471493</v>
       </c>
       <c r="N17" t="n">
-        <v>2.35572624790648e-06</v>
+        <v>-0.001507431665346373</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -1394,30 +1394,30 @@
         <v>0.5</v>
       </c>
       <c r="G18" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="H18" t="n">
         <v>0.1</v>
       </c>
       <c r="I18" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>sin(phi_Dp)sin(phi_kp)</t>
+          <t>ALL</t>
         </is>
       </c>
       <c r="K18" t="n">
         <v>100</v>
       </c>
       <c r="L18" t="n">
-        <v>-0.0001488455437843229</v>
+        <v>-0.03567178363475463</v>
       </c>
       <c r="M18" t="n">
-        <v>0.0005040356188673103</v>
+        <v>0.01017957012847935</v>
       </c>
       <c r="N18" t="n">
-        <v>-7.442277189216144e-06</v>
+        <v>-0.001783589181737732</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -1425,222 +1425,6 @@
         </is>
       </c>
       <c r="P18" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="B19" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="C19" t="n">
-        <v>1</v>
-      </c>
-      <c r="D19" t="n">
-        <v>100</v>
-      </c>
-      <c r="E19" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="F19" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G19" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="H19" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I19" t="n">
-        <v>50</v>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>sin(phi_Dp)sin(phi_kp)</t>
-        </is>
-      </c>
-      <c r="K19" t="n">
-        <v>100</v>
-      </c>
-      <c r="L19" t="n">
-        <v>-0.0003453369609816225</v>
-      </c>
-      <c r="M19" t="n">
-        <v>0.0007184779930692618</v>
-      </c>
-      <c r="N19" t="n">
-        <v>-1.726684804908113e-05</v>
-      </c>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>p</t>
-        </is>
-      </c>
-      <c r="P19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="B20" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="C20" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" t="n">
-        <v>100</v>
-      </c>
-      <c r="E20" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="F20" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G20" t="n">
-        <v>4</v>
-      </c>
-      <c r="H20" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I20" t="n">
-        <v>50</v>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>sin(phi_Dp)sin(phi_kp)</t>
-        </is>
-      </c>
-      <c r="K20" t="n">
-        <v>100</v>
-      </c>
-      <c r="L20" t="n">
-        <v>-0.0005240105555591238</v>
-      </c>
-      <c r="M20" t="n">
-        <v>0.001023477386483585</v>
-      </c>
-      <c r="N20" t="n">
-        <v>-2.620052777795619e-05</v>
-      </c>
-      <c r="O20" t="inlineStr">
-        <is>
-          <t>p</t>
-        </is>
-      </c>
-      <c r="P20" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="B21" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="C21" t="n">
-        <v>1</v>
-      </c>
-      <c r="D21" t="n">
-        <v>100</v>
-      </c>
-      <c r="E21" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="F21" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G21" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="H21" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I21" t="n">
-        <v>50</v>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>sin(phi_Dp)sin(phi_kp)</t>
-        </is>
-      </c>
-      <c r="K21" t="n">
-        <v>100</v>
-      </c>
-      <c r="L21" t="n">
-        <v>-0.000669038799970486</v>
-      </c>
-      <c r="M21" t="n">
-        <v>0.001419320114396683</v>
-      </c>
-      <c r="N21" t="n">
-        <v>-3.34519399985243e-05</v>
-      </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t>p</t>
-        </is>
-      </c>
-      <c r="P21" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="B22" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="C22" t="n">
-        <v>1</v>
-      </c>
-      <c r="D22" t="n">
-        <v>100</v>
-      </c>
-      <c r="E22" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="F22" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G22" t="n">
-        <v>5</v>
-      </c>
-      <c r="H22" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I22" t="n">
-        <v>50</v>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>sin(phi_Dp)sin(phi_kp)</t>
-        </is>
-      </c>
-      <c r="K22" t="n">
-        <v>100</v>
-      </c>
-      <c r="L22" t="n">
-        <v>-0.0007238728372346796</v>
-      </c>
-      <c r="M22" t="n">
-        <v>0.0018714884429574</v>
-      </c>
-      <c r="N22" t="n">
-        <v>-3.619364186173398e-05</v>
-      </c>
-      <c r="O22" t="inlineStr">
-        <is>
-          <t>p</t>
-        </is>
-      </c>
-      <c r="P22" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>